<commit_message>
docs: actualizar README, guía de contribución y Kanban
Refs: K-06
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://correo2urledu-my.sharepoint.com/personal/getoyom_correo_url_edu_gt/Documents/Sexto Semestre/Ingenieria de Software I/EDA proyecto/sistema-citas/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_98887390AAA25AFC294ACB30AF1A55969693A288" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A8A5AB4-9014-4999-951B-701B1A952822}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_98887390AAA25AFC294ACB30AF1A55969693A288" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D67A5FF-F840-468E-BE9F-CB4AB9E1A4E4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -739,7 +739,64 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -999,6 +1056,10 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1412,7 +1473,7 @@
         <v>17</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>130</v>
+        <v>18</v>
       </c>
       <c r="G6" s="8">
         <v>46308</v>
@@ -1542,7 +1603,7 @@
         <v>41</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G11" s="13">
         <v>46308</v>
@@ -1568,7 +1629,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G12" s="8">
         <v>46309</v>
@@ -1672,7 +1733,7 @@
         <v>60</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G16" s="8">
         <v>46308</v>
@@ -1802,7 +1863,7 @@
         <v>78</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G21" s="13">
         <v>46308</v>
@@ -1932,7 +1993,7 @@
         <v>85</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G26" s="8">
         <v>46308</v>
@@ -2129,6 +2190,25 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <conditionalFormatting sqref="F4:F33">
+    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="Completado">
+      <formula>NOT(ISERROR(SEARCH("Completado",F4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="En progreso">
+      <formula>NOT(ISERROR(SEARCH("En progreso",F4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="3" operator="containsText" text="En revisión">
+      <formula>NOT(ISERROR(SEARCH("En revisión",F4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="2" operator="containsText" text="En revisión">
+      <formula>NOT(ISERROR(SEARCH("En revisión",F4)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4:F34">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="En revisión">
+      <formula>NOT(ISERROR(SEARCH("En revisión",F4)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="F4:F33" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Backlog,Por hacer,En progreso,En revisión,Completado"</formula1>
@@ -2314,11 +2394,11 @@
       </c>
       <c r="B14" s="23">
         <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A14)</f>
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C14" s="24">
         <f>B14/$B$18</f>
-        <v>0.9</v>
+        <v>0.73333333333333328</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2327,11 +2407,11 @@
       </c>
       <c r="B15" s="23">
         <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A15)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="24">
         <f>B15/$B$18</f>
-        <v>3.3333333333333333E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2353,11 +2433,11 @@
       </c>
       <c r="B17" s="23">
         <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A17)</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C17" s="24">
         <f>B17/$B$18</f>
-        <v>3.3333333333333333E-2</v>
+        <v>0.23333333333333334</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
docs: actualizar Kanban con el estado final del proyecto
Refs: K-29
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://correo2urledu-my.sharepoint.com/personal/getoyom_correo_url_edu_gt/Documents/Sexto Semestre/Ingenieria de Software I/EDA proyecto/sistema-citas/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://correo2urledu-my.sharepoint.com/personal/getoyom_correo_url_edu_gt/Documents/Sexto Semestre/Ingenieria de Software I/EDA proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_98887390AAA25AFC294ACB30AF1A55969693A288" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D67A5FF-F840-468E-BE9F-CB4AB9E1A4E4}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="11_98887390AAA25AFC294ACB30AF1A55969693A288" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBB8E1A5-FD50-4BCF-B840-5247A2C59B88}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,9 @@
     <sheet name="Resumen y Métricas" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tablero Kanban'!$A$3:$H$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tablero Kanban'!$A$3:$H$32</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,12 +40,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="131">
   <si>
     <t>TABLERO KANBAN — PLANIFICACIÓN Y SEGUIMIENTO DE TAREAS</t>
   </si>
   <si>
-    <t>Total de tarjetas: 30  |  Módulos: M1 a M5 + Integración  |  Estado editable mediante lista desplegable</t>
+    <t>Total de tarjetas: 29  |  Módulos: M1 a M5 + Integración  |  Estado editable mediante lista desplegable</t>
   </si>
   <si>
     <t>ID</t>
@@ -75,7 +75,7 @@
     <t>K-05</t>
   </si>
   <si>
-    <t>Actualizar tedious a ≥ 20.3.6 (vulnerabilidad moderada en sprintf-js) cuando la versión tenga ≥ 2 semanas publicada</t>
+    <t>Actualizar dependencias con vulnerabilidades: tedious (sprintf-js), @azure/msal-node, body-parser y nodemailer</t>
   </si>
   <si>
     <t>Gabriel Toyom</t>
@@ -108,39 +108,39 @@
     <t>Levantar el entorno completo con docker compose up y documentar requisitos (RAM, puertos)</t>
   </si>
   <si>
+    <t>Los 8 contenedores quedan healthy o exited (0) (db-init) en la máquina de cada integrante</t>
+  </si>
+  <si>
+    <t>K-03</t>
+  </si>
+  <si>
+    <t>Revisar y defender la librería compartida: contrato de eventos, topología (quorum, DLX, delivery-limit) y cliente AMQP</t>
+  </si>
+  <si>
+    <t>RNF-01</t>
+  </si>
+  <si>
+    <t>Explica en 3 min por qué ack manual + quorum + DLX garantizan at-least-once</t>
+  </si>
+  <si>
+    <t>K-04</t>
+  </si>
+  <si>
+    <t>Pipeline CI en verde (lint, pruebas, npm audit, validación de compose)</t>
+  </si>
+  <si>
+    <t>Un PR con una prueba rota queda bloqueado</t>
+  </si>
+  <si>
+    <t>K-06</t>
+  </si>
+  <si>
+    <t>Guion del dry-run, reparto de quién habla y cronómetro (7–8 min)</t>
+  </si>
+  <si>
     <t>Por hacer</t>
   </si>
   <si>
-    <t>Los 8 contenedores quedan healthy o exited (0) (db-init) en la máquina de cada integrante</t>
-  </si>
-  <si>
-    <t>K-03</t>
-  </si>
-  <si>
-    <t>Revisar y defender la librería compartida: contrato de eventos, topología (quorum, DLX, delivery-limit) y cliente AMQP</t>
-  </si>
-  <si>
-    <t>RNF-01</t>
-  </si>
-  <si>
-    <t>Explica en 3 min por qué ack manual + quorum + DLX garantizan at-least-once</t>
-  </si>
-  <si>
-    <t>K-04</t>
-  </si>
-  <si>
-    <t>Pipeline CI en verde (lint, pruebas, npm audit, validación de compose)</t>
-  </si>
-  <si>
-    <t>Un PR con una prueba rota queda bloqueado</t>
-  </si>
-  <si>
-    <t>K-06</t>
-  </si>
-  <si>
-    <t>Guion del dry-run, reparto de quién habla y cronómetro (7–8 min)</t>
-  </si>
-  <si>
     <t>DEMO.md ensayado 2 veces dentro del tiempo</t>
   </si>
   <si>
@@ -399,18 +399,6 @@
     <t>Ensayo interno #2 cronometrado y video de respaldo de la demo</t>
   </si>
   <si>
-    <t>Demo en 7–8 min; video guardado por si falla la red o el equipo</t>
-  </si>
-  <si>
-    <t>K-30</t>
-  </si>
-  <si>
-    <t>Dry-run del Hito 2</t>
-  </si>
-  <si>
-    <t>Demo presentada y retroalimentación anotada como tarjetas nuevas</t>
-  </si>
-  <si>
     <t>RESUMEN EJECUTIVO — DISTRIBUCIÓN DE CARGA Y MÓDULOS</t>
   </si>
   <si>
@@ -439,6 +427,12 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>npm audit --omit=dev --audit-level=high sin vulnerabilidades y la demo funciona con Docker</t>
+  </si>
+  <si>
+    <t>Demo en video guardado por si falla la red o el equipo</t>
   </si>
 </sst>
 </file>
@@ -612,7 +606,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -632,9 +626,6 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -728,39 +719,18 @@
     <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -778,21 +748,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.59996337778862885"/>
+          <bgColor theme="0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -916,7 +872,7 @@
                   <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1056,10 +1012,6 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1345,9 +1297,31 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="5">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{3CB933C8-16C1-4E35-ADAB-698944EFF6DF}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;22741a15-51ec-4b00-9842-aec41646dde3&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1359,28 +1333,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
     </row>
     <row r="3" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1410,10 +1384,10 @@
     </row>
     <row r="4" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>12</v>
@@ -1421,47 +1395,51 @@
       <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="8">
-        <v>46321</v>
-      </c>
-      <c r="H4" s="4"/>
+      <c r="E4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="7">
+        <v>46307</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="A5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="13">
-        <v>46307</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>19</v>
+      <c r="F5" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="12">
+        <v>46308</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>12</v>
@@ -1470,50 +1448,50 @@
         <v>13</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="8">
-        <v>46308</v>
+        <v>25</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="7">
+        <v>46309</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="A7" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="13">
+      <c r="E7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="12">
         <v>46309</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>27</v>
+      <c r="H7" s="9" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>12</v>
@@ -1524,39 +1502,39 @@
       <c r="E8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" s="8">
-        <v>46309</v>
+      <c r="F8" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="7">
+        <v>46314</v>
       </c>
       <c r="H8" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="B9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="13">
+      <c r="F9" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="12">
         <v>46315</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="9" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1576,10 +1554,10 @@
       <c r="E10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="F10" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="7">
         <v>46311</v>
       </c>
       <c r="H10" s="4" t="s">
@@ -1587,28 +1565,28 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="13">
+      <c r="F11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="12">
         <v>46308</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="9" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1622,16 +1600,16 @@
       <c r="C12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="13" t="s">
         <v>40</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="8">
+      <c r="F12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="7">
         <v>46309</v>
       </c>
       <c r="H12" s="4" t="s">
@@ -1639,28 +1617,28 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G13" s="13">
+      <c r="F13" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="12">
         <v>46310</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="9" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1674,16 +1652,16 @@
       <c r="C14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="13" t="s">
         <v>40</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" s="8">
+      <c r="F14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="7">
         <v>46311</v>
       </c>
       <c r="H14" s="4" t="s">
@@ -1691,28 +1669,28 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F15" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="13">
+      <c r="F15" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="12">
         <v>46312</v>
       </c>
-      <c r="H15" s="10" t="s">
+      <c r="H15" s="9" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1726,16 +1704,16 @@
       <c r="C16" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="14" t="s">
         <v>59</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="8">
+      <c r="F16" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="7">
         <v>46308</v>
       </c>
       <c r="H16" s="4" t="s">
@@ -1743,28 +1721,28 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F17" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G17" s="13">
+      <c r="F17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="12">
         <v>46310</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="9" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1778,16 +1756,16 @@
       <c r="C18" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="14" t="s">
         <v>59</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F18" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" s="8">
+      <c r="F18" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="7">
         <v>46311</v>
       </c>
       <c r="H18" s="4" t="s">
@@ -1795,28 +1773,28 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19" s="13">
+      <c r="F19" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="12">
         <v>46311</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="9" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1830,16 +1808,16 @@
       <c r="C20" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="14" t="s">
         <v>59</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G20" s="8">
+      <c r="F20" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="7">
         <v>46312</v>
       </c>
       <c r="H20" s="4" t="s">
@@ -1847,28 +1825,28 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="F21" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G21" s="13">
+      <c r="F21" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="12">
         <v>46308</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="9" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1882,16 +1860,16 @@
       <c r="C22" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G22" s="8">
+      <c r="F22" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="7">
         <v>46310</v>
       </c>
       <c r="H22" s="4" t="s">
@@ -1899,28 +1877,28 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G23" s="13">
+      <c r="F23" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="12">
         <v>46311</v>
       </c>
-      <c r="H23" s="10" t="s">
+      <c r="H23" s="9" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1934,16 +1912,16 @@
       <c r="C24" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="16" t="s">
+      <c r="D24" s="15" t="s">
         <v>77</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G24" s="8">
+        <v>25</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" s="7">
         <v>46312</v>
       </c>
       <c r="H24" s="4" t="s">
@@ -1951,28 +1929,28 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D25" s="16" t="s">
+      <c r="D25" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" s="13">
+      <c r="E25" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="12">
         <v>46312</v>
       </c>
-      <c r="H25" s="10" t="s">
+      <c r="H25" s="9" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1986,16 +1964,16 @@
       <c r="C26" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="16" t="s">
         <v>96</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="F26" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G26" s="8">
+      <c r="F26" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26" s="7">
         <v>46308</v>
       </c>
       <c r="H26" s="4" t="s">
@@ -2003,28 +1981,28 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F27" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G27" s="13">
+      <c r="F27" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="12">
         <v>46309</v>
       </c>
-      <c r="H27" s="10" t="s">
+      <c r="H27" s="9" t="s">
         <v>100</v>
       </c>
     </row>
@@ -2038,16 +2016,16 @@
       <c r="C28" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="16" t="s">
         <v>96</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F28" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28" s="8">
+      <c r="F28" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G28" s="7">
         <v>46310</v>
       </c>
       <c r="H28" s="4" t="s">
@@ -2055,28 +2033,28 @@
       </c>
     </row>
     <row r="29" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E29" s="11" t="s">
+      <c r="E29" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="F29" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G29" s="13">
+      <c r="F29" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="12">
         <v>46311</v>
       </c>
-      <c r="H29" s="10" t="s">
+      <c r="H29" s="9" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2090,16 +2068,16 @@
       <c r="C30" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="17" t="s">
+      <c r="D30" s="16" t="s">
         <v>96</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30" s="8">
+        <v>25</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" s="7">
         <v>46312</v>
       </c>
       <c r="H30" s="4" t="s">
@@ -2107,28 +2085,28 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="F31" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G31" s="13">
+      <c r="F31" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" s="12">
         <v>46313</v>
       </c>
-      <c r="H31" s="10" t="s">
+      <c r="H31" s="9" t="s">
         <v>116</v>
       </c>
     </row>
@@ -2142,75 +2120,44 @@
       <c r="C32" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="17" t="s">
         <v>114</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="F32" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G32" s="8">
+      <c r="F32" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" s="7">
         <v>46315</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="C33" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="D33" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F33" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G33" s="13">
-        <v>46316</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H33" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:H32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:F33">
-    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="Completado">
-      <formula>NOT(ISERROR(SEARCH("Completado",F4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="En progreso">
-      <formula>NOT(ISERROR(SEARCH("En progreso",F4)))</formula>
-    </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" text="En revisión">
+  <conditionalFormatting sqref="F4:F32">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="En revisión">
       <formula>NOT(ISERROR(SEARCH("En revisión",F4)))</formula>
     </cfRule>
     <cfRule type="containsText" priority="2" operator="containsText" text="En revisión">
       <formula>NOT(ISERROR(SEARCH("En revisión",F4)))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F4:F34">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="En revisión">
-      <formula>NOT(ISERROR(SEARCH("En revisión",F4)))</formula>
+    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="En progreso">
+      <formula>NOT(ISERROR(SEARCH("En progreso",F4)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="Completado">
+      <formula>NOT(ISERROR(SEARCH("Completado",F4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F4:F33" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F4:F32" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Backlog,Por hacer,En progreso,En revisión,Completado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2229,226 +2176,226 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+    </row>
+    <row r="3" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="22">
+        <f>COUNTIF('Tablero Kanban'!$C$4:$C$32, A4)</f>
+        <v>7</v>
+      </c>
+      <c r="D4" s="23">
+        <f t="shared" ref="D4:D9" si="0">C4/$C$10</f>
+        <v>0.2413793103448276</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="26">
+        <f>COUNTIF('Tablero Kanban'!$C$4:$C$32, A5)</f>
+        <v>5</v>
+      </c>
+      <c r="D5" s="27">
+        <f t="shared" si="0"/>
+        <v>0.17241379310344829</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="22">
+        <f>COUNTIF('Tablero Kanban'!$C$4:$C$32, A6)</f>
+        <v>5</v>
+      </c>
+      <c r="D6" s="23">
+        <f t="shared" si="0"/>
+        <v>0.17241379310344829</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="26">
+        <f>COUNTIF('Tablero Kanban'!$C$4:$C$32, A7)</f>
+        <v>5</v>
+      </c>
+      <c r="D7" s="27">
+        <f t="shared" si="0"/>
+        <v>0.17241379310344829</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="22">
+        <f>COUNTIF('Tablero Kanban'!$C$4:$C$32, A8)</f>
+        <v>5</v>
+      </c>
+      <c r="D8" s="23">
+        <f t="shared" si="0"/>
+        <v>0.17241379310344829</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" s="26">
+        <f>COUNTIF('Tablero Kanban'!$C$4:$C$32, A9)</f>
+        <v>2</v>
+      </c>
+      <c r="D9" s="27">
+        <f t="shared" si="0"/>
+        <v>6.8965517241379309E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-    </row>
-    <row r="3" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="19" t="s">
+      <c r="B10" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="33">
+        <f>SUM(C4:C9)</f>
+        <v>29</v>
+      </c>
+      <c r="D10" s="34">
+        <f>SUM(D4:D9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C12" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D3" s="20" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="22">
+        <f>COUNTIF('Tablero Kanban'!$F$4:$F$32, A13)</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="23">
+        <f>B13/$B$18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="22">
+        <f>COUNTIF('Tablero Kanban'!$F$4:$F$32, A14)</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="23">
+        <f>B14/$B$18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="37" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="23">
-        <f>COUNTIF('Tablero Kanban'!$C$4:$C$33, A4)</f>
-        <v>7</v>
-      </c>
-      <c r="D4" s="24">
-        <f t="shared" ref="D4:D9" si="0">C4/$C$10</f>
-        <v>0.23333333333333334</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="27">
-        <f>COUNTIF('Tablero Kanban'!$C$4:$C$33, A5)</f>
-        <v>5</v>
-      </c>
-      <c r="D5" s="28">
-        <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="C6" s="23">
-        <f>COUNTIF('Tablero Kanban'!$C$4:$C$33, A6)</f>
-        <v>5</v>
-      </c>
-      <c r="D6" s="24">
-        <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="C7" s="27">
-        <f>COUNTIF('Tablero Kanban'!$C$4:$C$33, A7)</f>
-        <v>5</v>
-      </c>
-      <c r="D7" s="28">
-        <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" s="23">
-        <f>COUNTIF('Tablero Kanban'!$C$4:$C$33, A8)</f>
-        <v>5</v>
-      </c>
-      <c r="D8" s="24">
-        <f t="shared" si="0"/>
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="C9" s="27">
-        <f>COUNTIF('Tablero Kanban'!$C$4:$C$33, A9)</f>
-        <v>3</v>
-      </c>
-      <c r="D9" s="28">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
-        <v>127</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="34">
-        <f>SUM(C4:C9)</f>
-        <v>30</v>
-      </c>
-      <c r="D10" s="35">
-        <f>SUM(D4:D9)</f>
-        <v>0.99999999999999989</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>128</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="36" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="23">
-        <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A13)</f>
-        <v>1</v>
-      </c>
-      <c r="C13" s="24">
-        <f>B13/$B$18</f>
-        <v>3.3333333333333333E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="23">
-        <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A14)</f>
-        <v>22</v>
-      </c>
-      <c r="C14" s="24">
-        <f>B14/$B$18</f>
-        <v>0.73333333333333328</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="B15" s="23">
-        <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A15)</f>
+      <c r="B15" s="22">
+        <f>COUNTIF('Tablero Kanban'!$F$4:$F$32, A15)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="23">
         <f>B15/$B$18</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B16" s="23">
-        <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A16)</f>
+      <c r="A16" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" s="22">
+        <f>COUNTIF('Tablero Kanban'!$F$4:$F$32, A16)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="23">
         <f>B16/$B$18</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="23">
-        <f>COUNTIF('Tablero Kanban'!$F$4:$F$33, A17)</f>
-        <v>7</v>
-      </c>
-      <c r="C17" s="24">
+      <c r="A17" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="22">
+        <f>COUNTIF('Tablero Kanban'!$F$4:$F$32, A17)</f>
+        <v>29</v>
+      </c>
+      <c r="C17" s="23">
         <f>B17/$B$18</f>
-        <v>0.23333333333333334</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="33" t="s">
-        <v>132</v>
-      </c>
-      <c r="B18" s="34">
+      <c r="A18" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B18" s="33">
         <f>SUM(B13:B17)</f>
-        <v>30</v>
-      </c>
-      <c r="C18" s="35">
+        <v>29</v>
+      </c>
+      <c r="C18" s="34">
         <f>SUM(C13:C17)</f>
         <v>1</v>
       </c>

</xml_diff>